<commit_message>
prices and date updated
</commit_message>
<xml_diff>
--- a/Costi Bis Hotel.xlsx
+++ b/Costi Bis Hotel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mavitabile\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{75C0D49A-E207-4962-90BB-9E025FD84594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAA8EE98-C89A-4F82-941F-7A07E8D86100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2280" yWindow="2280" windowWidth="18720" windowHeight="11650" xr2:uid="{A8FB2AD8-F235-4970-A02D-E5CD62CF1199}"/>
   </bookViews>
@@ -440,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{619F0C14-B0DA-46B2-91D0-BB658E5A7997}">
-  <dimension ref="B2:D7"/>
+  <dimension ref="B2:E7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="18.7265625" bestFit="1" customWidth="1"/>
@@ -448,7 +448,7 @@
     <col min="4" max="4" width="12.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B2" s="2"/>
       <c r="C2" s="1" t="s">
         <v>5</v>
@@ -457,60 +457,65 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="3">
+        <v>79</v>
+      </c>
+      <c r="D3" s="3">
         <v>89</v>
       </c>
-      <c r="D3" s="3">
-        <v>79</v>
-      </c>
+      <c r="E3" s="3"/>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B4" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="3">
+        <v>89</v>
+      </c>
+      <c r="D4" s="3">
         <v>99</v>
       </c>
-      <c r="D4" s="3">
-        <v>89</v>
-      </c>
+      <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B5" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="3">
+        <v>115</v>
+      </c>
+      <c r="D5" s="3">
         <v>129</v>
       </c>
-      <c r="D5" s="3">
-        <v>115</v>
-      </c>
+      <c r="E5" s="3"/>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="3">
+        <v>139</v>
+      </c>
+      <c r="D6" s="3">
         <v>159</v>
       </c>
-      <c r="D6" s="3">
-        <v>139</v>
-      </c>
+      <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="3">
+        <v>169</v>
+      </c>
+      <c r="D7" s="3">
         <v>189</v>
       </c>
-      <c r="D7" s="3">
-        <v>169</v>
-      </c>
+      <c r="E7" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>